<commit_message>
Datos transaccionales: descarga del 26-10-2026 (cambios de estado en sep-oct)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oc-mensuales/articulos-de-aseo-e-higiene/oct-2026.xlsx
+++ b/docs/oc-mensuales/articulos-de-aseo-e-higiene/oct-2026.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M646"/>
+  <dimension ref="A1:M647"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -31526,7 +31526,7 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>1043046-111-CM26</t>
+          <t>1532192-50-CM26</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
@@ -31546,22 +31546,22 @@
       </c>
       <c r="E486" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F486" t="inlineStr">
         <is>
-          <t>62.000.450-2</t>
+          <t>69.071.000-5</t>
         </is>
       </c>
       <c r="G486" t="inlineStr">
         <is>
-          <t>DELEGACIÓN PRESIDENCIAL REGIONAL DE ÑUBLE</t>
+          <t>ILUSTRE MUNICIPALIDAD DE QUINTA NORMAL</t>
         </is>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I486" t="inlineStr">
@@ -31585,7 +31585,7 @@
         </is>
       </c>
       <c r="M486" s="2" t="n">
-        <v>873.58</v>
+        <v>1360.64</v>
       </c>
     </row>
     <row r="487">
@@ -31977,7 +31977,7 @@
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>1532192-50-CM26</t>
+          <t>1043046-111-CM26</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
@@ -31997,22 +31997,22 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F493" t="inlineStr">
         <is>
-          <t>69.071.000-5</t>
+          <t>62.000.450-2</t>
         </is>
       </c>
       <c r="G493" t="inlineStr">
         <is>
-          <t>ILUSTRE MUNICIPALIDAD DE QUINTA NORMAL</t>
+          <t>DELEGACIÓN PRESIDENCIAL REGIONAL DE ÑUBLE</t>
         </is>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I493" t="inlineStr">
@@ -32036,7 +32036,7 @@
         </is>
       </c>
       <c r="M493" s="2" t="n">
-        <v>1360.64</v>
+        <v>873.58</v>
       </c>
     </row>
     <row r="494">
@@ -32103,7 +32103,7 @@
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>607-331-CM26</t>
+          <t>838102-111-CM26</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
@@ -32128,32 +32128,32 @@
       </c>
       <c r="F495" t="inlineStr">
         <is>
-          <t>61.809.000-0</t>
+          <t>73.923.800-5</t>
         </is>
       </c>
       <c r="G495" t="inlineStr">
         <is>
-          <t>PARQUE METROPOLITANO DE SANTIAGO</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Tarapacá</t>
         </is>
       </c>
       <c r="I495" t="inlineStr">
         <is>
-          <t>DIMERC S A</t>
+          <t>COMERCIAL AGUSTIN LIMITADA</t>
         </is>
       </c>
       <c r="J495" t="inlineStr">
         <is>
-          <t>96.670.840-9</t>
+          <t>76.287.853-4</t>
         </is>
       </c>
       <c r="K495" t="inlineStr">
         <is>
-          <t>Antofagasta</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="L495" t="inlineStr">
@@ -32162,7 +32162,7 @@
         </is>
       </c>
       <c r="M495" s="2" t="n">
-        <v>34583.35</v>
+        <v>1646.26</v>
       </c>
     </row>
     <row r="496">
@@ -32615,7 +32615,7 @@
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>838102-111-CM26</t>
+          <t>607-331-CM26</t>
         </is>
       </c>
       <c r="B503" t="inlineStr">
@@ -32640,32 +32640,32 @@
       </c>
       <c r="F503" t="inlineStr">
         <is>
-          <t>73.923.800-5</t>
+          <t>61.809.000-0</t>
         </is>
       </c>
       <c r="G503" t="inlineStr">
         <is>
-          <t>DIVISION LOGISTICA DEL EJERCITO</t>
+          <t>PARQUE METROPOLITANO DE SANTIAGO</t>
         </is>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>Tarapacá</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I503" t="inlineStr">
         <is>
-          <t>COMERCIAL AGUSTIN LIMITADA</t>
+          <t>DIMERC S A</t>
         </is>
       </c>
       <c r="J503" t="inlineStr">
         <is>
-          <t>76.287.853-4</t>
+          <t>96.670.840-9</t>
         </is>
       </c>
       <c r="K503" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="L503" t="inlineStr">
@@ -32674,7 +32674,7 @@
         </is>
       </c>
       <c r="M503" s="2" t="n">
-        <v>1646.26</v>
+        <v>34583.35</v>
       </c>
     </row>
     <row r="504">
@@ -40006,7 +40006,7 @@
     <row r="618">
       <c r="A618" t="inlineStr">
         <is>
-          <t>2345-512-CM26</t>
+          <t>1622-1334-CM26</t>
         </is>
       </c>
       <c r="B618" t="inlineStr">
@@ -40031,43 +40031,47 @@
       </c>
       <c r="F618" t="inlineStr">
         <is>
-          <t>69.070.400-5</t>
+          <t>61.602.141-9</t>
         </is>
       </c>
       <c r="G618" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE LAS CONDES</t>
+          <t>SERVICIO DE SALUD HOSPITAL DE SAN VICENTE DE TAGUA TAGUA</t>
         </is>
       </c>
       <c r="H618" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I618" t="inlineStr">
         <is>
-          <t>LUIS ALEXANDER</t>
+          <t>MG PUBLICIDAD Y EVENTOS SPA</t>
         </is>
       </c>
       <c r="J618" t="inlineStr">
         <is>
-          <t>76.962.756-1</t>
-        </is>
-      </c>
-      <c r="K618" t="inlineStr"/>
+          <t>76.202.065-3</t>
+        </is>
+      </c>
+      <c r="K618" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L618" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
       <c r="M618" s="2" t="n">
-        <v>4647.93</v>
+        <v>3546.55</v>
       </c>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>1622-1334-CM26</t>
+          <t>2345-513-CM26</t>
         </is>
       </c>
       <c r="B619" t="inlineStr">
@@ -40092,27 +40096,27 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>61.602.141-9</t>
+          <t>69.070.400-5</t>
         </is>
       </c>
       <c r="G619" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD HOSPITAL DE SAN VICENTE DE TAGUA TAGUA</t>
+          <t>I MUNICIPALIDAD DE LAS CONDES</t>
         </is>
       </c>
       <c r="H619" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I619" t="inlineStr">
         <is>
-          <t>MG PUBLICIDAD Y EVENTOS SPA</t>
+          <t>CHICAUMA CHILE SPA</t>
         </is>
       </c>
       <c r="J619" t="inlineStr">
         <is>
-          <t>76.202.065-3</t>
+          <t>77.935.401-6</t>
         </is>
       </c>
       <c r="K619" t="inlineStr">
@@ -40126,7 +40130,7 @@
         </is>
       </c>
       <c r="M619" s="2" t="n">
-        <v>3546.55</v>
+        <v>22541.48</v>
       </c>
     </row>
     <row r="620">
@@ -40453,7 +40457,7 @@
     <row r="625">
       <c r="A625" t="inlineStr">
         <is>
-          <t>2345-513-CM26</t>
+          <t>2345-512-CM26</t>
         </is>
       </c>
       <c r="B625" t="inlineStr">
@@ -40493,26 +40497,22 @@
       </c>
       <c r="I625" t="inlineStr">
         <is>
-          <t>CHICAUMA CHILE SPA</t>
+          <t>LUIS ALEXANDER</t>
         </is>
       </c>
       <c r="J625" t="inlineStr">
         <is>
-          <t>77.935.401-6</t>
-        </is>
-      </c>
-      <c r="K625" t="inlineStr">
-        <is>
-          <t>Metropolitana</t>
-        </is>
-      </c>
+          <t>76.962.756-1</t>
+        </is>
+      </c>
+      <c r="K625" t="inlineStr"/>
       <c r="L625" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
       <c r="M625" s="2" t="n">
-        <v>22541.48</v>
+        <v>4647.93</v>
       </c>
     </row>
     <row r="626">
@@ -41099,7 +41099,7 @@
     <row r="635">
       <c r="A635" t="inlineStr">
         <is>
-          <t>359-3342-CM26</t>
+          <t>539119-3466-CM26</t>
         </is>
       </c>
       <c r="B635" t="inlineStr">
@@ -41124,12 +41124,12 @@
       </c>
       <c r="F635" t="inlineStr">
         <is>
-          <t>61.608.404-6</t>
+          <t>60.505.720-9</t>
         </is>
       </c>
       <c r="G635" t="inlineStr">
         <is>
-          <t>Instituto Nacional del Cancer</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H635" t="inlineStr">
@@ -41158,13 +41158,13 @@
         </is>
       </c>
       <c r="M635" s="2" t="n">
-        <v>1083.4</v>
+        <v>754.4299999999999</v>
       </c>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr">
         <is>
-          <t>2694-268-CM26</t>
+          <t>359-3342-CM26</t>
         </is>
       </c>
       <c r="B636" t="inlineStr">
@@ -41189,43 +41189,47 @@
       </c>
       <c r="F636" t="inlineStr">
         <is>
-          <t>69.073.600-4</t>
+          <t>61.608.404-6</t>
         </is>
       </c>
       <c r="G636" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE CARTAGENA</t>
+          <t>Instituto Nacional del Cancer</t>
         </is>
       </c>
       <c r="H636" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I636" t="inlineStr">
         <is>
-          <t>GRULLA SPA</t>
+          <t>PROVEEDORES INTEGRALES PRISA S A</t>
         </is>
       </c>
       <c r="J636" t="inlineStr">
         <is>
-          <t>77.235.846-6</t>
-        </is>
-      </c>
-      <c r="K636" t="inlineStr"/>
+          <t>96.556.940-5</t>
+        </is>
+      </c>
+      <c r="K636" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L636" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
       <c r="M636" s="2" t="n">
-        <v>2169.82</v>
+        <v>1083.4</v>
       </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
         <is>
-          <t>545598-989-CM26</t>
+          <t>2694-268-CM26</t>
         </is>
       </c>
       <c r="B637" t="inlineStr">
@@ -41250,47 +41254,43 @@
       </c>
       <c r="F637" t="inlineStr">
         <is>
-          <t>71.149.700-5</t>
+          <t>69.073.600-4</t>
         </is>
       </c>
       <c r="G637" t="inlineStr">
         <is>
-          <t>CORP MUNICIPAL DE CASTRO PARA LA EDUCACION SALUD Y ATENCION AL MENOR</t>
+          <t>I MUNICIPALIDAD DE CARTAGENA</t>
         </is>
       </c>
       <c r="H637" t="inlineStr">
         <is>
-          <t>Los Lagos</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I637" t="inlineStr">
         <is>
-          <t>PROVEEDORES INTEGRALES PRISA S A</t>
+          <t>GRULLA SPA</t>
         </is>
       </c>
       <c r="J637" t="inlineStr">
         <is>
-          <t>96.556.940-5</t>
-        </is>
-      </c>
-      <c r="K637" t="inlineStr">
-        <is>
-          <t>Metropolitana</t>
-        </is>
-      </c>
+          <t>77.235.846-6</t>
+        </is>
+      </c>
+      <c r="K637" t="inlineStr"/>
       <c r="L637" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
       <c r="M637" s="2" t="n">
-        <v>8302.32</v>
+        <v>2169.82</v>
       </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
         <is>
-          <t>3117-1499-CM26</t>
+          <t>545598-989-CM26</t>
         </is>
       </c>
       <c r="B638" t="inlineStr">
@@ -41315,43 +41315,47 @@
       </c>
       <c r="F638" t="inlineStr">
         <is>
-          <t>61.102.006-6</t>
+          <t>71.149.700-5</t>
         </is>
       </c>
       <c r="G638" t="inlineStr">
         <is>
-          <t>DIRECCION DE ABASTECIMIENTO DE LA ARMADA</t>
+          <t>CORP MUNICIPAL DE CASTRO PARA LA EDUCACION SALUD Y ATENCION AL MENOR</t>
         </is>
       </c>
       <c r="H638" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I638" t="inlineStr">
         <is>
-          <t>SOCIEDAD COMERCIAL MEGASTORE LIMITADA</t>
+          <t>PROVEEDORES INTEGRALES PRISA S A</t>
         </is>
       </c>
       <c r="J638" t="inlineStr">
         <is>
-          <t>76.935.880-3</t>
-        </is>
-      </c>
-      <c r="K638" t="inlineStr"/>
+          <t>96.556.940-5</t>
+        </is>
+      </c>
+      <c r="K638" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L638" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
       <c r="M638" s="2" t="n">
-        <v>2658.79</v>
+        <v>8302.32</v>
       </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
         <is>
-          <t>1725-1066-CM26</t>
+          <t>3117-1499-CM26</t>
         </is>
       </c>
       <c r="B639" t="inlineStr">
@@ -41376,12 +41380,12 @@
       </c>
       <c r="F639" t="inlineStr">
         <is>
-          <t>60.901.002-9</t>
+          <t>61.102.006-6</t>
         </is>
       </c>
       <c r="G639" t="inlineStr">
         <is>
-          <t>SUBSECRETARÍA DE LAS CULTURAS Y LAS ARTES</t>
+          <t>DIRECCION DE ABASTECIMIENTO DE LA ARMADA</t>
         </is>
       </c>
       <c r="H639" t="inlineStr">
@@ -41391,26 +41395,22 @@
       </c>
       <c r="I639" t="inlineStr">
         <is>
-          <t>EVENTAIL SPA</t>
+          <t>SOCIEDAD COMERCIAL MEGASTORE LIMITADA</t>
         </is>
       </c>
       <c r="J639" t="inlineStr">
         <is>
-          <t>76.710.414-6</t>
-        </is>
-      </c>
-      <c r="K639" t="inlineStr">
-        <is>
-          <t>Metropolitana</t>
-        </is>
-      </c>
+          <t>76.935.880-3</t>
+        </is>
+      </c>
+      <c r="K639" t="inlineStr"/>
       <c r="L639" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
       <c r="M639" s="2" t="n">
-        <v>7061.08</v>
+        <v>2658.79</v>
       </c>
     </row>
     <row r="640">
@@ -41481,7 +41481,7 @@
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t>5060-930-CM26</t>
+          <t>4819-128-CM26</t>
         </is>
       </c>
       <c r="B641" t="inlineStr">
@@ -41506,27 +41506,27 @@
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>69.190.700-7</t>
+          <t>60.201.000-7</t>
         </is>
       </c>
       <c r="G641" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE TEMUCO</t>
+          <t>SENADO DE LA REPUBLICA</t>
         </is>
       </c>
       <c r="H641" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I641" t="inlineStr">
         <is>
-          <t>COMERCIAL AGUSTIN LIMITADA</t>
+          <t>PROVEEDORES INTEGRALES PRISA S A</t>
         </is>
       </c>
       <c r="J641" t="inlineStr">
         <is>
-          <t>76.287.853-4</t>
+          <t>96.556.940-5</t>
         </is>
       </c>
       <c r="K641" t="inlineStr">
@@ -41540,13 +41540,13 @@
         </is>
       </c>
       <c r="M641" s="2" t="n">
-        <v>903.6799999999999</v>
+        <v>1286.3</v>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
         <is>
-          <t>2111-13070-CM26</t>
+          <t>5060-930-CM26</t>
         </is>
       </c>
       <c r="B642" t="inlineStr">
@@ -41571,27 +41571,27 @@
       </c>
       <c r="F642" t="inlineStr">
         <is>
-          <t>61.608.602-2</t>
+          <t>69.190.700-7</t>
         </is>
       </c>
       <c r="G642" t="inlineStr">
         <is>
-          <t>HOSPITAL DE URGENCIA ASISTENCIA PUBLICA DR ALEJANDRO DEL RIO</t>
+          <t>I MUNICIPALIDAD DE TEMUCO</t>
         </is>
       </c>
       <c r="H642" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I642" t="inlineStr">
         <is>
-          <t>MG PUBLICIDAD Y EVENTOS SPA</t>
+          <t>COMERCIAL AGUSTIN LIMITADA</t>
         </is>
       </c>
       <c r="J642" t="inlineStr">
         <is>
-          <t>76.202.065-3</t>
+          <t>76.287.853-4</t>
         </is>
       </c>
       <c r="K642" t="inlineStr">
@@ -41605,13 +41605,13 @@
         </is>
       </c>
       <c r="M642" s="2" t="n">
-        <v>5784.87</v>
+        <v>903.6799999999999</v>
       </c>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>4778-579-CM26</t>
+          <t>2111-13070-CM26</t>
         </is>
       </c>
       <c r="B643" t="inlineStr">
@@ -41636,43 +41636,47 @@
       </c>
       <c r="F643" t="inlineStr">
         <is>
-          <t>61.602.280-6</t>
+          <t>61.608.602-2</t>
         </is>
       </c>
       <c r="G643" t="inlineStr">
         <is>
-          <t>SERVICIO NACIONAL DE SALUD HOSPITAL DE C</t>
+          <t>HOSPITAL DE URGENCIA ASISTENCIA PUBLICA DR ALEJANDRO DEL RIO</t>
         </is>
       </c>
       <c r="H643" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I643" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA Y COMERCIAL DIMAK LIMITADA</t>
+          <t>MG PUBLICIDAD Y EVENTOS SPA</t>
         </is>
       </c>
       <c r="J643" t="inlineStr">
         <is>
-          <t>78.809.560-0</t>
-        </is>
-      </c>
-      <c r="K643" t="inlineStr"/>
+          <t>76.202.065-3</t>
+        </is>
+      </c>
+      <c r="K643" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L643" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
       <c r="M643" s="2" t="n">
-        <v>28432.24</v>
+        <v>5784.87</v>
       </c>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>539119-3466-CM26</t>
+          <t>4778-579-CM26</t>
         </is>
       </c>
       <c r="B644" t="inlineStr">
@@ -41697,47 +41701,43 @@
       </c>
       <c r="F644" t="inlineStr">
         <is>
-          <t>60.505.720-9</t>
+          <t>61.602.280-6</t>
         </is>
       </c>
       <c r="G644" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>SERVICIO NACIONAL DE SALUD HOSPITAL DE C</t>
         </is>
       </c>
       <c r="H644" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I644" t="inlineStr">
         <is>
-          <t>PROVEEDORES INTEGRALES PRISA S A</t>
+          <t>DISTRIBUIDORA Y COMERCIAL DIMAK LIMITADA</t>
         </is>
       </c>
       <c r="J644" t="inlineStr">
         <is>
-          <t>96.556.940-5</t>
-        </is>
-      </c>
-      <c r="K644" t="inlineStr">
-        <is>
-          <t>Metropolitana</t>
-        </is>
-      </c>
+          <t>78.809.560-0</t>
+        </is>
+      </c>
+      <c r="K644" t="inlineStr"/>
       <c r="L644" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
       <c r="M644" s="2" t="n">
-        <v>754.4299999999999</v>
+        <v>28432.24</v>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
         <is>
-          <t>4819-128-CM26</t>
+          <t>4493-745-CM26</t>
         </is>
       </c>
       <c r="B645" t="inlineStr">
@@ -41762,27 +41762,27 @@
       </c>
       <c r="F645" t="inlineStr">
         <is>
-          <t>60.201.000-7</t>
+          <t>69.150.502-2</t>
         </is>
       </c>
       <c r="G645" t="inlineStr">
         <is>
-          <t>SENADO DE LA REPUBLICA</t>
+          <t>I MUNICIPALIDAD DE PENCO</t>
         </is>
       </c>
       <c r="H645" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I645" t="inlineStr">
         <is>
-          <t>PROVEEDORES INTEGRALES PRISA S A</t>
+          <t>COMERCIAL MUNOZ Y COMPANIA LIMITADA</t>
         </is>
       </c>
       <c r="J645" t="inlineStr">
         <is>
-          <t>96.556.940-5</t>
+          <t>78.906.980-8</t>
         </is>
       </c>
       <c r="K645" t="inlineStr">
@@ -41796,13 +41796,13 @@
         </is>
       </c>
       <c r="M645" s="2" t="n">
-        <v>1286.3</v>
+        <v>1423.11</v>
       </c>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr">
         <is>
-          <t>4493-745-CM26</t>
+          <t>1725-1066-CM26</t>
         </is>
       </c>
       <c r="B646" t="inlineStr">
@@ -41827,27 +41827,27 @@
       </c>
       <c r="F646" t="inlineStr">
         <is>
-          <t>69.150.502-2</t>
+          <t>60.901.002-9</t>
         </is>
       </c>
       <c r="G646" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE PENCO</t>
+          <t>SUBSECRETARÍA DE LAS CULTURAS Y LAS ARTES</t>
         </is>
       </c>
       <c r="H646" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I646" t="inlineStr">
         <is>
-          <t>COMERCIAL MUNOZ Y COMPANIA LIMITADA</t>
+          <t>EVENTAIL SPA</t>
         </is>
       </c>
       <c r="J646" t="inlineStr">
         <is>
-          <t>78.906.980-8</t>
+          <t>76.710.414-6</t>
         </is>
       </c>
       <c r="K646" t="inlineStr">
@@ -41861,7 +41861,68 @@
         </is>
       </c>
       <c r="M646" s="2" t="n">
-        <v>1423.11</v>
+        <v>7061.08</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>1422824-3436-CM26</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>2239-8-LR25</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>oct-2026</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Aceptada</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>61.602.054-4</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>SERVICIO NACIONAL DE SALUD HOSPITAL CARLOS VAN BUREN</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>Valparaíso</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>Proser S.A.</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>76.308.616-k</t>
+        </is>
+      </c>
+      <c r="K647" t="inlineStr"/>
+      <c r="L647" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M647" s="2" t="n">
+        <v>52859.17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>